<commit_message>
Add new image files for project assets
- Added 'minkalab.jpg' to the raw image assets.
- Added 'sustratos_colombia.jpg' to the raw image assets.
- Added 'termales_ruiz.png' to the raw image assets.
</commit_message>
<xml_diff>
--- a/raw/actores.xlsx
+++ b/raw/actores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brian.amaya\Documents\2.Proyectos\TNC\talleres_regionales\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76DA0057-4011-4739-91FB-3B29FCC8B4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98EB3197-A3ED-45B6-BBD1-3C2BA6A71F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="28800" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="organizaciones" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="401">
   <si>
     <t>organización</t>
   </si>
@@ -499,9 +499,6 @@
     <t>hacienda el bosque sas</t>
   </si>
   <si>
-    <t>yuliana.cruz@udea.edu.co</t>
-  </si>
-  <si>
     <t>5.066979767689393, -75.51824580346957</t>
   </si>
   <si>
@@ -509,6 +506,756 @@
   </si>
   <si>
     <t>5.045436552988614, -75.51197293230574</t>
+  </si>
+  <si>
+    <t>Hacienda Charrascal</t>
+  </si>
+  <si>
+    <t>Nuestra organización integra turismo rural, patrimonio cultural cafetero, gastronomía tradicional y sostenibilidad ambiental a través de experiencias que promueven el aprovechamiento responsable de los recursos naturales y culturales del territorio. Desde Hacienda Charrascal y Fogón de Palo impulsamos prácticas relacionadas con la bioeconomía mediante el turismo sostenible, la valorización del café y los productos locales, la conservación del paisaje cultural cafetero, el fortalecimiento de economías rurales y la generación de experiencias educativas y culturales conectadas con la biodiversidad y las tradiciones campesinas.</t>
+  </si>
+  <si>
+    <t>Patrimonio – Sostenibilidad – Turismo</t>
+  </si>
+  <si>
+    <t>https://haciendacharrascal.co/</t>
+  </si>
+  <si>
+    <t>5.133308468072525, -75.50106369778496</t>
+  </si>
+  <si>
+    <t>charrascal.jpg</t>
+  </si>
+  <si>
+    <t>Hotel Termales del Ruiz</t>
+  </si>
+  <si>
+    <t>Hotel Termales del Ruiz integra prácticas de turismo sostenible enfocadas en el aprovechamiento responsable de los recursos naturales y el bienestar ambiental. La organización promueve experiencias de ecoturismo y bienestar alrededor de los ecosistemas de alta montaña y las aguas termales, impulsando la conservación ambiental, el uso eficiente de recursos, la educación ambiental y el desarrollo sostenible del territorio mediante actividades turísticas basadas en la biodiversidad y los servicios ecosistémicos de la región.</t>
+  </si>
+  <si>
+    <t>Turismo – Bienestar – Sostenibilidad</t>
+  </si>
+  <si>
+    <t>https://termalesdelruiz.com/</t>
+  </si>
+  <si>
+    <t>4.970529390345127, -75.37822837403061</t>
+  </si>
+  <si>
+    <t>termales_ruiz.png</t>
+  </si>
+  <si>
+    <t>minkalab.org</t>
+  </si>
+  <si>
+    <t>MinkaLab impulsa iniciativas de bioeconomía a través de la producción agroecológica, la transformación de productos agrícolas, el turismo rural y las experiencias educativas basadas en la biodiversidad local. Trabajamos en la regeneración de ecosistemas y suelos, promoviendo modelos productivos que generan valor económico a partir del uso sostenible de los recursos biológicos y los conocimientos tradicionales. Además, fortalecemos capacidades comunitarias mediante procesos de intercambio de saberes, innovación social y desarrollo de emprendimientos que contribuyen al bienestar de las personas y la conservación del territorio.</t>
+  </si>
+  <si>
+    <t>Regeneración - Cultura - Innovación Social</t>
+  </si>
+  <si>
+    <t>www.minkalab.org</t>
+  </si>
+  <si>
+    <t>4.876603920093241, -75.6046299554575</t>
+  </si>
+  <si>
+    <t>minkalab.jpg</t>
+  </si>
+  <si>
+    <t>Arcesio Holguín Orozco</t>
+  </si>
+  <si>
+    <t>Filósofo y especialista en sostenibilidad y nuevas economías. Actualmente lidero procesos comerciales y de posicionamiento territorial en Hacienda Charrascal y Fogón de Palo, articulando alianzas entre empresa, cultura y comunidad. Además, soy creador de SUMÁNDONOS, una iniciativa de innovación social enfocada en sostenibilidad, reconciliación ambiental y trabajo comunitario. Interesado en la bioeconomía, las nuevas economías y el desarrollo territorial sostenible.</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/arcesio-holguín-41a178142</t>
+  </si>
+  <si>
+    <t>arcesio.holguin@gmail.com</t>
+  </si>
+  <si>
+    <t>Representante Legal</t>
+  </si>
+  <si>
+    <t>Kely Dahiana Gutiérrez Patiño</t>
+  </si>
+  <si>
+    <t>Consultora en implementación, acompañamiento y certificación de sistemas de gestión en calidad, sostenibilidad y seguridad y salud en el trabajo.</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/kelly__dahiana/?hl=es</t>
+  </si>
+  <si>
+    <t>calidad@hotelcarretero.com</t>
+  </si>
+  <si>
+    <t>Lider de Gestión Integral y desarrollo sostenible</t>
+  </si>
+  <si>
+    <t>Inversiones GFL S.A</t>
+  </si>
+  <si>
+    <t>Gabriel Vanegas</t>
+  </si>
+  <si>
+    <t>Gabriel Vanegas es emprendedor social, facilitador de procesos comunitarios y cofundador de MinkaLab, un laboratorio vivo orientado a la regeneración territorial, el intercambio de saberes y la innovación social. Su trabajo integra agroecología, turismo consciente, educación experiencial y desarrollo comunitario, promoviendo iniciativas que fortalecen la relación entre las personas, la cultura y la naturaleza. Cuenta con experiencia en el diseño y gestión de proyectos de impacto social, ambiental y cultural, así como en la creación de experiencias de aprendizaje vinculadas al buen vivir y la sostenibilidad.</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/minkalabcolombia/</t>
+  </si>
+  <si>
+    <t>info@minkalab.org</t>
+  </si>
+  <si>
+    <t>director</t>
+  </si>
+  <si>
+    <t>Yuliana.cruz@udea.edu.co</t>
+  </si>
+  <si>
+    <t>Brian Amaya</t>
+  </si>
+  <si>
+    <t>Economista con experiencia en bioeconomía, competitividad y desarrollo económico, especializado en la creación de métricas e 
+indicadores para el análisis y seguimiento de indicadores socioeconómicos. Cuento con habilidades sólidas en el manejo e 
+interpretación de datos multidisciplinarios, enfocados en encadenamientos productivos y desarrollo sostenible a escala territorial. Mi 
+trayectoria abarca el uso de tecnologías 4.0 para el diseño de herramientas analíticas que optimizan procesos y apoyan la toma de 
+decisiones estratégicas en los territorios</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/brianamaya01</t>
+  </si>
+  <si>
+    <t>bamaya@humboldt.org.co</t>
+  </si>
+  <si>
+    <t>Bogotá D.C.</t>
+  </si>
+  <si>
+    <t>Investigador</t>
+  </si>
+  <si>
+    <t>Instituto Humboldt</t>
+  </si>
+  <si>
+    <t>Olga Lucia Ocampo López</t>
+  </si>
+  <si>
+    <t>Doctora en Ingeniería. Coordinadora del Doctorado en Sostenibilidad de la Universidad Autónoma de Manizales. Profesora titular. investigadora Senior</t>
+  </si>
+  <si>
+    <t>@olgaocampolopez</t>
+  </si>
+  <si>
+    <t>olocampo@autonoma.edu.co</t>
+  </si>
+  <si>
+    <t>Coordinadora Doctorado en Sostenibilidad</t>
+  </si>
+  <si>
+    <t>Luz Piedad Romero Duque</t>
+  </si>
+  <si>
+    <t>Doctorado en ciencias biológicas de la UNAM. Líneas biodiversidad y servicios ecosistémicos, ciencias ambientales.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/luz-piedad-romero-duque-phd-83b31533</t>
+  </si>
+  <si>
+    <t>Luz.romero@jbotanico.org</t>
+  </si>
+  <si>
+    <t>Directora de Investigación</t>
+  </si>
+  <si>
+    <t>Jardín Botánico de Medellin</t>
+  </si>
+  <si>
+    <t>Kelly Orozco</t>
+  </si>
+  <si>
+    <t>Biologa, Magister en Ciencias Biológicas y estudiante Doctorado en Estudios Territoriales de la Universidad de Caldas. Con experiencia en Ornitología , conservación , aviturismo, educación ambiental y trabajo comunitario. Actualmente directora de la Reserva Metamorfosis</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>kellyorozco@fcvcol.org</t>
+  </si>
+  <si>
+    <t>Directora Reserva Metamorfosis</t>
+  </si>
+  <si>
+    <t>Fundación para la Conservación de la Vida Silvestre en Colombia</t>
+  </si>
+  <si>
+    <t>Juan Sebastian Blandón Rendón</t>
+  </si>
+  <si>
+    <t>Cocreador del proyecto de agroecologia y Permacultura ecofinca la soledad, productores de plantas medicinales con certificación orgánica y transformadores.</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/ecofincalasoledad?igsh=MTVydG5hZWF3bnllaQ==</t>
+  </si>
+  <si>
+    <t>ecofincalasoledade91@gmail.com</t>
+  </si>
+  <si>
+    <t>Sonia Pardo</t>
+  </si>
+  <si>
+    <t>Ingeniera Forestal con MSc en Agricultura Internacional Sostenible, trabajo en The Nature Conservancy como Especialista en Soluciones Basadas en la Naturaleza para Mitigación. Lidero la línea de trabajo en bioeconomía, apoyando el diseño e implementación de estrategias de bioeconomía en la Amazonía Andina. Mi trabajo se centra en conectar la conservación, la producción sostenible y las oportunidades económicas para impulsar soluciones prácticas basadas en la naturaleza. Me motiva colaborar con actores de distintos sectores para convertir ideas en redes y alianzas que aporten a la conservación y a mejores oportunidades económicas para las personas y el país.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/sonia-pardo-guti%C3%A9rrez-/</t>
+  </si>
+  <si>
+    <t>sonia.pardo@tnc.org</t>
+  </si>
+  <si>
+    <t>Especialista en Soluciones basadas en la Naturaleza para la Mitigación del Cambio Climático</t>
+  </si>
+  <si>
+    <t>The Nature Conservancy</t>
+  </si>
+  <si>
+    <t>Carlos Alberto López Cañas</t>
+  </si>
+  <si>
+    <t>Especialista en gestión ambiental y magíster en gestión tecnológica. Trayectoria de 21 años en formulación, gestión y ejecución de proyectos de CTeI con empresas privadas, entidades públicas y organizaciones de cooperación nacional e internacional.</t>
+  </si>
+  <si>
+    <t>https://co.linkedin.com/in/carlos-a-l%C3%B3pez-c-1243b622?trk=people-guest_people_search-card</t>
+  </si>
+  <si>
+    <t>carlos.lopezcanas@antioquia.gov.co</t>
+  </si>
+  <si>
+    <t>Profesional especializado</t>
+  </si>
+  <si>
+    <t>Gobernación de Antioquia</t>
+  </si>
+  <si>
+    <t>Juan Carlos Parra Espitia</t>
+  </si>
+  <si>
+    <t>Especialista en Planeación Integrada para la Conservación, The Nature Conservancy (TNC). Area de trabajo bioeconomía con experiencia en amazonia andina y Orinoquia.</t>
+  </si>
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>juan.parra@tnc.org</t>
+  </si>
+  <si>
+    <t>Guaviare</t>
+  </si>
+  <si>
+    <t>Especialista en Planeación Integrada para la conservacion.</t>
+  </si>
+  <si>
+    <t>Jhon Fredy Betancur Perez</t>
+  </si>
+  <si>
+    <t>Docente Investigador - Universidad de Manizales</t>
+  </si>
+  <si>
+    <t>Instagram</t>
+  </si>
+  <si>
+    <t>jbetancur@umanizales.edu.co</t>
+  </si>
+  <si>
+    <t>Carlos David Muñoz Ortiz</t>
+  </si>
+  <si>
+    <t>Administrador de empresas especializado en Alta Gerencia, mi recorrido profesional ha sido en la Cámara de Comercio de Manizales por Caldas, trabajé aportando al fortalecimiento del sector empresarial turístico y actualmente me desempeño como profesional de la Comisión Regional de Competitividad e Innovación de Caldas articulando actores del ecosistema de competitividad y gestionando proyectos en la Agenda Departamental de Competitividad e Innovación de Caldas.</t>
+  </si>
+  <si>
+    <t>https://co.linkedin.com/in/carlos-david-munoz-ortiz-910865307</t>
+  </si>
+  <si>
+    <t>crcicaldas@ccm.org.co</t>
+  </si>
+  <si>
+    <t>Profesional de la CRCI Caldas</t>
+  </si>
+  <si>
+    <t>Comisión Regional de Competitividad e Innovación de Caldas</t>
+  </si>
+  <si>
+    <t>Julián Mauricio Calle Aguirre</t>
+  </si>
+  <si>
+    <t>Apicultor y caficultor, pionero en el occidente de Risaralda y Caldas en agroindustria Apícola y del Café, especialista en agroturísmo, cultural e histórico y turismo de naturaleza. Administrador de Empresas Agropecuarias y Medio Ambiente, Guía Profesional de Turismo y Magister en Desarrollo Sostenible y Medio Ambiente.</t>
+  </si>
+  <si>
+    <t>Facebook: Apícola del Viento Apia</t>
+  </si>
+  <si>
+    <t>mauriapi@gmail.com</t>
+  </si>
+  <si>
+    <t>Fundador, director y líder de operaciones</t>
+  </si>
+  <si>
+    <t>Asociación Agropecuaria y Agroindustrial Apícola del Viento APIVIEN y Bicitours Rutas del Viento</t>
+  </si>
+  <si>
+    <t>Adriana Bolaños Mora</t>
+  </si>
+  <si>
+    <t>Doctora y Magíster en Diseño por la Universidad Federal do Rio Grande do Sul, Especialista en Mercadeo y Diseñadora Gráfica por la Universidad del Cauca. Mi trayectoria integra la investigación, la creación y la gestión de proyectos orientados al diseño y la educación. Soy investigadora de Plantas Alimenticias Nativas No Convencionales (PANNC), diseñadora de maletas didácticas y promotora de iniciativas que articulan conocimiento, territorio y cultura. Además de mi labor académica y profesional, soy mamá y cocinera empírica, experiencias que enriquecen mi mirada sobre el diseño como herramienta para la transformación social.</t>
+  </si>
+  <si>
+    <t>@pannc.colombia</t>
+  </si>
+  <si>
+    <t>adrianabmora@gmail.com</t>
+  </si>
+  <si>
+    <t>Quindío</t>
+  </si>
+  <si>
+    <t>Jardín Botánico del Quindío</t>
+  </si>
+  <si>
+    <t>Héctor Favio Manrique Fierro</t>
+  </si>
+  <si>
+    <t>Ingeniero Agroecólogo, MSc en Gestión y Auditorias Ambientales, Director General del Jardín Botánico del Quindío, curador de la Colección de Palmas de Colombia.</t>
+  </si>
+  <si>
+    <t>agroecologo.ua@gmail.com</t>
+  </si>
+  <si>
+    <t>Director General</t>
+  </si>
+  <si>
+    <t>Maria Alejandrs Cuervo Cardona</t>
+  </si>
+  <si>
+    <t>Administradora de empresas, especialista en gerencia de proyectos con formación complementaria en metodologías de creatividad e innovación, emprendimiento de base tecnológica, vigilancia tecnológica, tecnología exponenciales. Con más de 12 años de experiencia en el sector de Ciencia Tecnología e Innovación, actualmente trabajo para la Gobernación de Caldas - Secretaría de Desarrollo Empleo e Innovación con la implementación y puesta en operación del Parque Científico Tecnológico y de Innovación de Caldas FUTURA.</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/maria-alejandra-cuervo-cardona</t>
+  </si>
+  <si>
+    <t>macuervocc@gobernaciondecaldas.gov.co</t>
+  </si>
+  <si>
+    <t>Asesora proyectos especiales Unidad de CTeI - Secretaría de Desarrollo Empleo e Innovación - Gobernación de Caldas</t>
+  </si>
+  <si>
+    <t>Gobernación de Caldas</t>
+  </si>
+  <si>
+    <t>Alejandro Arango</t>
+  </si>
+  <si>
+    <t>Economista con un perfil de emprendedor en un proyecto de gestión ambiental de residuos sólidos orgánicos de la industria de manizales</t>
+  </si>
+  <si>
+    <t>LinkedIn Facebook Instagram</t>
+  </si>
+  <si>
+    <t>Alear00@hotmail.com</t>
+  </si>
+  <si>
+    <t>Gerente de ventas</t>
+  </si>
+  <si>
+    <t>Sustratos de Colombia</t>
+  </si>
+  <si>
+    <t>Juliana Arias Villegas</t>
+  </si>
+  <si>
+    <t>Administradora Ambiental, estudiante del Doctorado en Biotecnología y miembro del grupo de investigación Biodiversidad y Biotecnología de la Universidad Tecnológica de Pereira.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/juliana-arias-villegas-620302141/</t>
+  </si>
+  <si>
+    <t>juliana@utp.edu.co</t>
+  </si>
+  <si>
+    <t>Profesional líder Gestión Tecnológica, Innovación y Emprendimiento de la Vicerrectoría de Investigaciones, Innovación y Extensión</t>
+  </si>
+  <si>
+    <t>Universidad Tecnológica de Pereira</t>
+  </si>
+  <si>
+    <t>Daniela López Montoya</t>
+  </si>
+  <si>
+    <t>Sociologa estudiante PhD en Medioambiente y Sociedad</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/daniela-lopez-montoya/</t>
+  </si>
+  <si>
+    <t>proyectos.provinciacartama@gmail.com</t>
+  </si>
+  <si>
+    <t>Lider de proyectos y gestión de alianzas</t>
+  </si>
+  <si>
+    <t>Provincia De Administración Y Planificación Cartama</t>
+  </si>
+  <si>
+    <t>Juan Carlos Zuluaga Cardona</t>
+  </si>
+  <si>
+    <t>Magister Administración de Negocios</t>
+  </si>
+  <si>
+    <t>juancarloszuluagacardona@gmail.com</t>
+  </si>
+  <si>
+    <t>Gerente</t>
+  </si>
+  <si>
+    <t>Bank of tierras de Colombia</t>
+  </si>
+  <si>
+    <t>Leonidas Robledo Sanchez</t>
+  </si>
+  <si>
+    <t>Geologo Magister en Saneamiento y Desarrollo Ambiental, con énfasis y amplia experiencia en gestión del riesgo y estudios de impacto ambiental</t>
+  </si>
+  <si>
+    <t>Linkedin</t>
+  </si>
+  <si>
+    <t>leonidasrobledo@gmail.com</t>
+  </si>
+  <si>
+    <t>Sinergia Ambiental Colombia S.A.S</t>
+  </si>
+  <si>
+    <t>Ximena Carranza Hernandez</t>
+  </si>
+  <si>
+    <t>Bióloga especialista en planeación ambiental y manejo integral de los recursos naturales, con más de 10 años de experiencia en el sector público en el área ambiental, con énfasis en la gestión integral de la biodiversidad y sus servicios ecosistémicos para el desarrollo de bienes y servicios que impulsen la bioeconomía colombiana, así como la construcción, evaluación y seguimiento a las políticas públicas, planes, programas, estrategias e instrumentos de uso sostenible de la biodiversidad. Mi experiencia también abarca la investigación en ecología de ambientes acuáticos, trayectoria en docencia y formación profesional para el trabajo.</t>
+  </si>
+  <si>
+    <t>linkedin.com/in/ximenacarranzahernandez</t>
+  </si>
+  <si>
+    <t>xcarranza@dnp.gov.co</t>
+  </si>
+  <si>
+    <t>Contratista</t>
+  </si>
+  <si>
+    <t>Departamento Nacional de Planeación (DNP)</t>
+  </si>
+  <si>
+    <t>Maria Camila Aguirre Arroyave</t>
+  </si>
+  <si>
+    <t>Soy Ingeniera en procesos Agroindustriales egresada de la UTP y actualmente trabajo como ejecutiva comercial de una empresa comercializadora de equipos para laboratorios</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/maria-camila-aguirre-arroyave-087982325?utm_source=share_via&amp;utm_content=profile&amp;utm_medium=member_android</t>
+  </si>
+  <si>
+    <t>Maguirre@intekgroup.com.co</t>
+  </si>
+  <si>
+    <t>Ejecutiva comercial</t>
+  </si>
+  <si>
+    <t>Intek Group</t>
+  </si>
+  <si>
+    <t>Angie Mondragón</t>
+  </si>
+  <si>
+    <t>Economista, Magister en Economía, PhD (c) en Economía</t>
+  </si>
+  <si>
+    <t>https://co.linkedin.com/in/angie-alejandra-mondrag%C3%B3n-mayo-709679ab</t>
+  </si>
+  <si>
+    <t>amondragon@humboldt.org.co</t>
+  </si>
+  <si>
+    <t>Gobierno departamental de Caldas, con jurisdicción sobre 27 municipios en la región del Eje Cafetero colombiano. La Secretaría de Desarrollo, Empleo e Innovación es la dependencia que articuló la participación de la Gobernación en el ecosistema bioeconómico del departamento.
+- Coejecutora del Programa Biofábricas (MinCiencias, 2022-2024): participó en los tres proyectos-misión del programa junto con la Universidad-de-Manizales y otras instituciones.
+- Miembro activo de la Mision-de-Sabios-Caldas(2020-2021), que estableció las líneas estratégicas de CTeI + educación para el departamento y fue la incubadora del Programa Biofábricas.
+- Caldas fue el primer departamento colombiano en implementar los acuerdos de la Misión Internacional de Sabios 2019.
+- Desde la Secretaría de Desarrollo, Empleo e Innovación, articula actores universitarios, comunitarios e institucionales para el modelo bioeconómico territorial.</t>
+  </si>
+  <si>
+    <t>Gobernanza - Desarrollo - Parque Tecnológico</t>
+  </si>
+  <si>
+    <t>https://caldas.gov.co/</t>
+  </si>
+  <si>
+    <t>https://brianamaya01.github.io/biolink_col/wiki/entities/Gobernacion-Caldas</t>
+  </si>
+  <si>
+    <t>5.06873022451919, -75.51748613558209</t>
+  </si>
+  <si>
+    <t>Biointropic</t>
+  </si>
+  <si>
+    <t>Biointropic acompaña negocios, empresas y proyectos de base bioinnovadora en los sectores cosméticos, alimentos y agro. Facilita conexiones de valor y sinergias entre empresas, academia y gobierno para el desarrollo de bioproductos.
+- Elabora el Portafolio de Ingredientes Naturales (BIO IN) de Colombia, referencia clave del ecosistema de ingredientes naturales nacional, que presenta 12 empresas ancla vinculadas a los sectores de cosmética, aseo, alimentos, bebidas y químico.
+- Publicó el estudio "Bioeconomía como fuente de nuevas industrias basadas en el capital natural de Colombia" (2018), que contribuyó a la definición oficial de bioeconomía en el CONPES 3934.
+- En alianza con el DNP publicó **"BIOECONOMÍA Y SECTORES"** (2018): documento de referencia del sector biotech nacional — base de datos y clasificación utilizada en múltiples estudios posteriores.
+- Realizó en **2017** el primer mapeo sistemático de empresas biotech en Colombia: **203 empresas** registradas que elaboran productos derivados de investigación en biodiversidad. Distribución: 39% biotecnología verde, 35% biotecnología blanca (industrial), 19% salud (roja), 7% gris. El **77%** de estas empresas se concentra en Antioquia, Bogotá y Valle del Cauca.</t>
+  </si>
+  <si>
+    <t>Ingredientes naturales - Cosmética - Alimentos</t>
+  </si>
+  <si>
+    <t>https://biointropic.com/</t>
+  </si>
+  <si>
+    <t>https://brianamaya01.github.io/biolink_col/wiki/entities/Biointropic</t>
+  </si>
+  <si>
+    <t>6.2027925502290575, -75.57252318418065</t>
+  </si>
+  <si>
+    <t>biointropic.jpg</t>
+  </si>
+  <si>
+    <t>En la Provincia Cartama del suroeste antioqueño se ha avanzado significativamente en bioeconomía mediante el Laboratorio de Innovación en Bioeconomía instalado en mayo de 2025 en el Agroparque Biosuroeste de Támesis, donde 42 entidades de gobierno, academia, empresa y comunidad colaboraron para definir cinco líneas productivas estratégicas: agropecuario, agroindustrial (café, cacao, cítricos), uso sostenible de bosques, turismo de naturaleza y bioproductos de alto valor, dentro de una estrategia articulada por la Provincia de Administración y Planificación Cartama con Fundación Con Vida y el apoyo del Fondo de Alianzas para los Ecosistemas Críticos (CEPF) y el Gobierno de Canadá a través de la iniciativa "Cultivadores de Biodiversidad" que incluye 16 bioemprendimientos locales, ocho liderados por mujeres, dedicados a cafés especiales, productos apícolas, turismo de naturaleza y agroturismo, complementado con la reciente trazación en febrero de 2026 de la Ruta de Bioeconomía para el Turismo, experiencias emblemáticas como el Laboratorio de Café de Támesis, Ecotransformemos con biotecnología para biofertilizantes, Frudelca con economía circular en cítricos, y la Ruta de Bioeconomía para la Paz en Santa Bárbara, todo ello enmarcado en la Ruta Cartama Sostenible 2030 que articula 31 proyectos de protección de ecosistemas y producción responsable en once municipios, posicionando al territorio como un modelo de desarrollo regenerativo que conecta biodiversidad, conocimiento científico y comunidad.</t>
+  </si>
+  <si>
+    <t>Bioemprendimientos - Uso sostenible - Turismo de naturaleza</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/provinciacartama/</t>
+  </si>
+  <si>
+    <t>5.621822782264991, -75.69936234871636</t>
+  </si>
+  <si>
+    <t>cartama.jpg</t>
+  </si>
+  <si>
+    <t>En la Universidad Tecnológica de Pereira (UTP) se han desarrollado múltiples iniciativas vinculadas a la bioeconomía: en 2023, la universidad, junto con las Cátedras UNESCO y el IICA, ofreció el Diplomado Internacional en Bioeconomía Aplicada a la Cadena de Valor del Café (90 horas, modalidad virtual), Dirigido a productores, emprendedores y estudiantes de 15 países de América Latina, con becas del 100% y enfoque en aprovechamiento sostenible de biomasa y transformación de recursos biológicos en bioproductos y bioservicios; también en 2023, la UTP albergó el II Foro Regional de Bioeconomía liderado por la RAP Eje Cafetero, con representantes de Caldas, Quindío, Tolima y Risaralda, donde se presentaron proyectos de cuatro cadenas de valor priorizadas (aguacate, café, cacao y plátano), sistemas de información e investigaciones, con conferencia magistral de la experta Elizabeth Hodson y recorrido por el Centro de Desarrollo Tecnológico Agroindustrial (CDTA), que cuenta con 17 laboratorios equipados para investigación y generación de productos de valor agregado; la universidad organiza desde 2019 el Congreso Internacional de Biotecnología y Bioeconomía</t>
+  </si>
+  <si>
+    <t>Formación-Diplomados-Biomasa</t>
+  </si>
+  <si>
+    <t>https://www.utp.edu.co/</t>
+  </si>
+  <si>
+    <t>4.795535127725845, -75.68772606675013</t>
+  </si>
+  <si>
+    <t>UTP.png</t>
+  </si>
+  <si>
+    <t>El Jardín Botánico del Quindío, ubicado en Calarcá, ha consolidado iniciativas clave vinculadas a la conservación y uso sostenible de la biodiversidad, con aplicaciones directas en bioeconomía: fue fundado en 1979 por Alberto Gómez Mejía como el primer jardín botánico legal de Colombia y originalmente concebido como centro de investigación para conservación ecológica; alberga la colección de palmeras más grande del país, junto con colecciones botánicas nativas de Palmae, Heliconia, Pteridofitos (helechos), Lauráceas, Orquidáceas, Bromeliáceas y Aráceas, además de plantas medicinales, carnívoras y especies en peligro de extinción; cuenta con el Mariposario (uno de sus principales atractivos ecoturísticos) donde habitan alrededor de 1.500 mariposas de 40-50 especies volando libremente, el Insectario, el Bosque de Colibríes, un puente colgante, el Guadual, el Jardín de los Enamorados, el Laberinto, el Museo de Geología y Suelos, el Mapa 3D del Quindío, y programas de avistamiento de aves; promete turismo de naturaleza y educación ambiental como ejes de bioeconomía circular al conectar biodiversidad, conocimiento científico y experiencia turística; en febrero 2026, reforzó su alianza estratégica con la Universidad del Quindío mediante un convenio de cooperación que articula educación ambiental, investigación aplicada y apropiación social del conocimiento, articulando la Facultad de Ciencias Básicas y Tecnologías y el Centro de Investigaciones en Biodiversidad (CIBUQ) en la estructuración del Diplomado en Conservación, Uso y Manejo de la Biodiversidad con módulos en botánica aplicada, áreas de conservación, fauna regional, política pública, divulgación científica y química de metabolitos secundarios, proyectando que los participantes desarrollen proyectos de investigación aplicada en el jardín como laboratorio vivo; el jardín funciona como laboratorio vivo para investigación y educación ambiental con respaldo científico universitario para la conservación del patrimonio natural del Quindío y el Eje Cafetero</t>
+  </si>
+  <si>
+    <t>Educación ambiental-Uso sostenible de la biodiversidad-Turismo de naturaleza</t>
+  </si>
+  <si>
+    <t>https://jardinbotanicoquindio.org/</t>
+  </si>
+  <si>
+    <t>4.511915898417822, -75.65103621302856</t>
+  </si>
+  <si>
+    <t>jardin-quindio.png</t>
+  </si>
+  <si>
+    <t>El Instituto de Investigación de Recursos Biológicos Alexander von Humboldt (Instituto Humboldt) investiga y promueve el conocimiento, la conservación y el uso sostenible de la biodiversidad en Colombia. Impulsa la bioprospección, el uso sostenible de la biodiversidad y modelos de negocio basados en recursos biológicos.
+Promueve la generación de alternativas económicas sostenibles en comunidades locales y apoya la conservación ambiental, articulando ciencia, sostenibilidad y desarrollo productivo. 
+Investiga y desarrolla tecnologías que transfiere a productores locales para innovar y generar mayores ingresos. 
+Fomenta productos alimenticios con valor nutricional y beneficios adicionales para la salud, aprovechando la biodiversidad local.</t>
+  </si>
+  <si>
+    <t>Biodiversidad - Bioeconomía - Cadenas de valor</t>
+  </si>
+  <si>
+    <t>https://www.humboldt.org.co/</t>
+  </si>
+  <si>
+    <t>https://brianamaya01.github.io/biolink_col/wiki/entities/Instituto-Humboldt</t>
+  </si>
+  <si>
+    <t>4.664255062065658, -74.06271471035458</t>
+  </si>
+  <si>
+    <t>Humboldt-logo.jpg</t>
+  </si>
+  <si>
+    <t>El Jardín Botánico de Medellín es una institución líder en conservación de la biodiversidad, investigación científica, educación ambiental y gestión del conocimiento sobre los recursos biológicos de Colombia. Su trabajo contribuye al fortalecimiento de la bioeconomía mediante la generación de conocimiento sobre especies nativas, restauración ecológica y aprovechamiento responsable de la biodiversidad. Buscamos desarrollar esta línea de investigación con énfasis en seguridad alimentaria, promoviendo soluciones basadas en la biodiversidad que fortalezcan sistemas productivos sostenibles, la conservación de los recursos naturales y el bienestar de las comunidades.</t>
+  </si>
+  <si>
+    <t>Conservación-investigación-educación de plantas</t>
+  </si>
+  <si>
+    <t>https://www.botanicomedellin.org/</t>
+  </si>
+  <si>
+    <t>6.2695417931117365, -75.56490861301594</t>
+  </si>
+  <si>
+    <t>jardin-medellin.png</t>
+  </si>
+  <si>
+    <t>La Fundación para la Conservación de la Vida Silvestre en Colombia es una organización con más de tres décadas de experiencia dedicada a la conservación de la biodiversidad y la gestión sostenible del territorio. Su trabajo integra investigación, conservación de ecosistemas, fortalecimiento de reservas naturales, agroecología, turismo científico y participación comunitaria, promoviendo la conectividad ecológica entre paisajes productivos y áreas protegidas. Entre sus iniciativas destacan la Agenda de Montaña y el Mosaico de Conservación Arma–Miel, estrategias orientadas a la protección de corredores biológicos, la gobernanza ambiental y el desarrollo sostenible de las regiones andinas. Buscamos desarrollar esta línea de investigación con énfasis en seguridad alimentaria, impulsando modelos de producción agroecológica, conservación de la biodiversidad y aprovechamiento sostenible de los recursos naturales que contribuyan al bienestar de las comunidades rurales y a la resiliencia de los territorios.</t>
+  </si>
+  <si>
+    <t>Conservación-Gobernanza-Territorio</t>
+  </si>
+  <si>
+    <t>https://fcvcol.org/</t>
+  </si>
+  <si>
+    <t>5.38446894204548, -75.16161711913213</t>
+  </si>
+  <si>
+    <t>fundacion_conservacion_vida_silvestre.png</t>
+  </si>
+  <si>
+    <t>La The Nature Conservancy es una organización global de conservación que promueve modelos de desarrollo sostenible basados en la protección de la biodiversidad, el uso responsable de los recursos naturales y la generación de oportunidades económicas para las comunidades. En Colombia, TNC impulsa iniciativas relacionadas con la bioeconomía, las soluciones basadas en la naturaleza, la producción sostenible, la restauración de ecosistemas y la seguridad alimentaria, buscando que la conservación y el desarrollo económico avancen de manera conjunta. Su trabajo integra ciencia, innovación y alianzas con gobiernos, empresas y comunidades para fortalecer cadenas de valor sostenibles que aprovechen la biodiversidad como motor de desarrollo regional. Buscamos desarrollar esta línea de investigación con énfasis en seguridad alimentaria, promoviendo el aprovechamiento sostenible de la biodiversidad, la producción agropecuaria regenerativa y la generación de bio-negocios que contribuyan a la conservación de los ecosistemas y al bienestar de las comunidades rurales</t>
+  </si>
+  <si>
+    <t>Cambio Climático-Bioeconomía-Trabajo con Comunidades y Pueblos Indigenas</t>
+  </si>
+  <si>
+    <t>https://www.nature.org/es-us/sobre-tnc/donde-trabajamos/tnc-en-latinoamerica/colombia/</t>
+  </si>
+  <si>
+    <t>4.651628952303022, -74.0587537246699</t>
+  </si>
+  <si>
+    <t>The-Nature-Conservancy.jpg</t>
+  </si>
+  <si>
+    <t>La Gobernación de Antioquia es el órgano de gobierno del departamento de Antioquia, el segundo motor económico de Colombia (14,4 % del PIB nacional). Está compuesta por múltiples secretarías; las más relevantes para la bioeconomía son la Secretaría de Productividad y Competitividad (a cargo de la estrategia de bioeconomía), la Secretaría de Ambiente y Sostenibilidad y la Secretaría de Agricultura y Desarrollo Rural. Maneja una de las autonomías fiscales más altas del país (36,7 %) y administra los recursos del Sistema General de Regalías (SGR) para CTeI en el departamento.
+En 2023, la Gobernación —a través de la Secretaría de Productividad y Competitividad (liderada por Daniela Trejo Rojas)— elaboró junto con el GGGI la “Aproximación a la Estrategia Bioeconomía para Antioquia”, el primer documento estratégico del departamento en esta materia. La estrategia plantea 4 líneas estratégicas (gobernanza, capacidades tecnológicas, gestión de recursos económicos, sostenibilidad social y ambiental), 10 brechas identificadas y un modelo de gobernanza tripartito.</t>
+  </si>
+  <si>
+    <t>Desarrollo - comunidad - sostenibilidad</t>
+  </si>
+  <si>
+    <t>https://co.linkedin.com/company/gobantioquia</t>
+  </si>
+  <si>
+    <t>https://brianamaya01.github.io/biolink_col/wiki/entities/Gobernacion-Antioquia</t>
+  </si>
+  <si>
+    <t>6.244204581414633, -75.57362050359801</t>
+  </si>
+  <si>
+    <t>gob_antioquia.jpg</t>
+  </si>
+  <si>
+    <t>La Comisión Regional de Competitividad e Innovación de Caldas es una instancia de articulación entre los sectores público, privado, académico y social que promueve estrategias para fortalecer la competitividad, la innovación y el desarrollo sostenible del departamento. A través de la dinamización de mesas temáticas, la Comisión impulsa procesos orientados al cierre de brechas territoriales, la generación de capacidades y la construcción de agendas colaborativas para el desarrollo económico regional. En este contexto, la mesa de economía circular se constituye como un espacio clave para fomentar el uso eficiente de los recursos, la innovación empresarial y la transición hacia modelos productivos más sostenibles. Buscamos desarrollar esta línea de investigación con énfasis en seguridad alimentaria, promoviendo la economía circular aplicada a los sistemas agroalimentarios, el aprovechamiento de biomasa y residuos orgánicos, y la generación de soluciones innovadoras que fortalezcan la sostenibilidad y resiliencia de los territorios.</t>
+  </si>
+  <si>
+    <t>Competitividad-Territorialización-Proyectos</t>
+  </si>
+  <si>
+    <t>www.crcicaldas.com</t>
+  </si>
+  <si>
+    <t>5.0399060432157885, -75.4468554995326</t>
+  </si>
+  <si>
+    <t>crci-caldas.jpg</t>
+  </si>
+  <si>
+    <t>Movemos mesas temáticas entorno a cierre de brechas en este caso tenemos mesa de economía circular en el territorio.</t>
+  </si>
+  <si>
+    <t>5.105798620175925, -75.9396140048931</t>
+  </si>
+  <si>
+    <t>apicola-asociacion-viento-apia.jpg</t>
+  </si>
+  <si>
+    <t>Creamos abono #orgánico que nutre el suelo, fortalece los cultivos y protege el futuro del planeta.
+Desarrollamos productos para la agricultura a base de biotecnología aplicada al campo</t>
+  </si>
+  <si>
+    <t>Bioeconomia-agricultura-gestión ambiental</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/sustratosdecolombia/</t>
+  </si>
+  <si>
+    <t>5.008010576810856, -75.4395248265181</t>
+  </si>
+  <si>
+    <t>sustratos_colombia.jpg</t>
+  </si>
+  <si>
+    <t>Es una plataforma donde usted, su familia o empresa, compensan el daño que todos causamos al planeta, a través de la adopción de árboles y metros cuadrados de tierra en común y proindiviso, para la protección de la flora, la fauna, el agua y todas las formas de vida que subsista en los ecosistemas que protegemos, asegurando la acción climática como una oportunidad para los adoptantes y las entidades gubernamentales.</t>
+  </si>
+  <si>
+    <t>Bioprospeccion</t>
+  </si>
+  <si>
+    <t>https://www.bankoftierras.com/</t>
+  </si>
+  <si>
+    <t>5.070228640040919, -75.62045179325128</t>
+  </si>
+  <si>
+    <t>bank_of_tierras.jpg</t>
+  </si>
+  <si>
+    <t>Diseño y desarrollo de proyectos en manejo de residuos sólidos, vertimientos y suministro de agua</t>
+  </si>
+  <si>
+    <t>Medio Ambiente, urbanismo y bioeconomia</t>
+  </si>
+  <si>
+    <t>El Departamento Nacional de Planeación (DNP) es la entidad gubernamental responsable de la planeación y orientación de políticas públicas de largo plazo en Colombia. Define marcos de política económica, social y ambiental, incluyendo los documentos CONPES y el Plan Nacional de Desarrollo. Coordina la Dirección de Ambiente y Desarrollo Sostenible (DADS), que lidera la agenda de transición ecológica y bioeconomía.
+El DNP ha sido actor central en la institucionalización de la bioeconomía en Colombia: 
+Estudio fundacional (2018): “Estudio sobre la bioeconomía como fuente de nuevas industrias basadas en el capital natural de Colombia” — primer análisis técnico nacional que posicionó la bioeconomía como estrategia de desarrollo. 
+Misión de Crecimiento Verde (2015-2018): coordinó el acopio de información sobre capacidades y necesidades en aprovechamiento de biodiversidad y biomasa. 
+CONPES 3934 (2018): Política de Crecimiento Verde, que incluye la bioeconomía como eje estratégico. 
+CONPES 4129 (2023): Política Nacional de Reindustrialización, con mandato de 32 agendas departamentales de bioeconomía. 
+Transición ecológica: La DADS definió la transición ecológica como “el proceso para acelerar la transformación justa del modelo económico actual, a uno con estándares de crecimiento más resilientes y sostenibles haciendo uso eficiente del capital natural.” 
+Producto Ecosistémico Bruto (PEB): El DNP promueve métricas complementarias al PIB que incluyan el capital natural como activo estratégico de la nación, en coordinación con el DANE. 
+Cooperación con Natural Capital Project (Stanford): modelamiento de servicios ecosistémicos (protección costera, carbono azul, oferta hídrica) como base para planificación territorial. 
+Potencial empleo bioecónomico (DNP/OIT, 2020)</t>
+  </si>
+  <si>
+    <t>Bioeconomía-Planificación Territorial</t>
+  </si>
+  <si>
+    <t>http://www.dnp.gov.co</t>
+  </si>
+  <si>
+    <t>https://brianamaya01.github.io/biolink_col/wiki/entities/DNP</t>
+  </si>
+  <si>
+    <t>4.613257759169303, -74.0717775490756</t>
+  </si>
+  <si>
+    <t>dnp.jpg</t>
+  </si>
+  <si>
+    <t>Empresa colombiana dedicada a la distribución de equipos especializados para laboratorio y maquinaria industrial, brindando soluciones pertinentes, efectivas y rentables mediante el uso de últimas tecnologías de información y comunicación. Poniendo a su disposición un equipo técnico de expertos altamente capacitado para ayudar a encontrar las soluciones apropiadas que su organización necesita. 
+Intek ha desarrollado un importante reconocimiento en el campo de la biotecnología y bioprocesos, así como convertirse en un actor de referencia en el suministro de sistemas de microscopía de alta resolución que contribuyen a la construcción nanotecnología dentro del campo de la caracterización de materiales, basados siempre en un gran compromiso para ofertar soluciones optimas a nuestros clientes.</t>
+  </si>
+  <si>
+    <t>Biotecnología-Equipos-Laboratorios</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/company/intek-group-sas/?originalSubdomain=co</t>
+  </si>
+  <si>
+    <t>intek_group_sas_logo.jpg</t>
   </si>
 </sst>
 </file>
@@ -566,10 +1313,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -851,13 +1599,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -880,7 +1628,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -903,7 +1651,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -923,7 +1671,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -943,7 +1691,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -963,7 +1711,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -980,7 +1728,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -1003,7 +1751,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>41</v>
       </c>
@@ -1020,7 +1768,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -1034,13 +1782,13 @@
         <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -1054,13 +1802,13 @@
         <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>56</v>
       </c>
@@ -1074,13 +1822,13 @@
         <v>59</v>
       </c>
       <c r="F11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G11" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -1100,24 +1848,424 @@
         <v>66</v>
       </c>
     </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" t="s">
+        <v>163</v>
+      </c>
+      <c r="F13" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B14" t="s">
+        <v>167</v>
+      </c>
+      <c r="C14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F14" t="s">
+        <v>170</v>
+      </c>
+      <c r="G14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" t="s">
+        <v>173</v>
+      </c>
+      <c r="C15" t="s">
+        <v>174</v>
+      </c>
+      <c r="D15" t="s">
+        <v>175</v>
+      </c>
+      <c r="F15" t="s">
+        <v>176</v>
+      </c>
+      <c r="G15" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>272</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C16" t="s">
+        <v>318</v>
+      </c>
+      <c r="D16" t="s">
+        <v>319</v>
+      </c>
+      <c r="E16" t="s">
+        <v>320</v>
+      </c>
+      <c r="F16" t="s">
+        <v>321</v>
+      </c>
+      <c r="G16" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>322</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="C17" t="s">
+        <v>324</v>
+      </c>
+      <c r="D17" t="s">
+        <v>325</v>
+      </c>
+      <c r="E17" t="s">
+        <v>326</v>
+      </c>
+      <c r="F17" t="s">
+        <v>327</v>
+      </c>
+      <c r="G17" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>290</v>
+      </c>
+      <c r="B18" t="s">
+        <v>329</v>
+      </c>
+      <c r="C18" t="s">
+        <v>330</v>
+      </c>
+      <c r="D18" t="s">
+        <v>331</v>
+      </c>
+      <c r="F18" t="s">
+        <v>332</v>
+      </c>
+      <c r="G18" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>284</v>
+      </c>
+      <c r="B19" t="s">
+        <v>334</v>
+      </c>
+      <c r="C19" t="s">
+        <v>335</v>
+      </c>
+      <c r="D19" t="s">
+        <v>336</v>
+      </c>
+      <c r="F19" t="s">
+        <v>337</v>
+      </c>
+      <c r="G19" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>262</v>
+      </c>
+      <c r="B20" t="s">
+        <v>339</v>
+      </c>
+      <c r="C20" t="s">
+        <v>340</v>
+      </c>
+      <c r="D20" t="s">
+        <v>341</v>
+      </c>
+      <c r="F20" t="s">
+        <v>342</v>
+      </c>
+      <c r="G20" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>201</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="C21" t="s">
+        <v>345</v>
+      </c>
+      <c r="D21" t="s">
+        <v>346</v>
+      </c>
+      <c r="E21" t="s">
+        <v>347</v>
+      </c>
+      <c r="F21" t="s">
+        <v>348</v>
+      </c>
+      <c r="G21" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>212</v>
+      </c>
+      <c r="B22" t="s">
+        <v>350</v>
+      </c>
+      <c r="C22" t="s">
+        <v>351</v>
+      </c>
+      <c r="D22" t="s">
+        <v>352</v>
+      </c>
+      <c r="F22" t="s">
+        <v>353</v>
+      </c>
+      <c r="G22" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B23" t="s">
+        <v>355</v>
+      </c>
+      <c r="C23" t="s">
+        <v>356</v>
+      </c>
+      <c r="D23" t="s">
+        <v>357</v>
+      </c>
+      <c r="F23" t="s">
+        <v>358</v>
+      </c>
+      <c r="G23" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" t="s">
+        <v>360</v>
+      </c>
+      <c r="C24" t="s">
+        <v>361</v>
+      </c>
+      <c r="D24" t="s">
+        <v>362</v>
+      </c>
+      <c r="F24" t="s">
+        <v>363</v>
+      </c>
+      <c r="G24" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>234</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="C25" t="s">
+        <v>366</v>
+      </c>
+      <c r="D25" t="s">
+        <v>367</v>
+      </c>
+      <c r="E25" t="s">
+        <v>368</v>
+      </c>
+      <c r="F25" t="s">
+        <v>369</v>
+      </c>
+      <c r="G25" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>250</v>
+      </c>
+      <c r="B26" t="s">
+        <v>371</v>
+      </c>
+      <c r="C26" t="s">
+        <v>372</v>
+      </c>
+      <c r="D26" t="s">
+        <v>373</v>
+      </c>
+      <c r="F26" t="s">
+        <v>374</v>
+      </c>
+      <c r="G26" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>256</v>
+      </c>
+      <c r="B27" t="s">
+        <v>376</v>
+      </c>
+      <c r="C27" t="s">
+        <v>372</v>
+      </c>
+      <c r="D27" t="s">
+        <v>373</v>
+      </c>
+      <c r="F27" t="s">
+        <v>377</v>
+      </c>
+      <c r="G27" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>278</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C28" t="s">
+        <v>380</v>
+      </c>
+      <c r="D28" t="s">
+        <v>381</v>
+      </c>
+      <c r="F28" t="s">
+        <v>382</v>
+      </c>
+      <c r="G28" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>295</v>
+      </c>
+      <c r="B29" t="s">
+        <v>384</v>
+      </c>
+      <c r="C29" t="s">
+        <v>385</v>
+      </c>
+      <c r="D29" t="s">
+        <v>386</v>
+      </c>
+      <c r="F29" t="s">
+        <v>387</v>
+      </c>
+      <c r="G29" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>300</v>
+      </c>
+      <c r="B30" t="s">
+        <v>389</v>
+      </c>
+      <c r="C30" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>306</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="C31" t="s">
+        <v>392</v>
+      </c>
+      <c r="D31" t="s">
+        <v>393</v>
+      </c>
+      <c r="E31" t="s">
+        <v>394</v>
+      </c>
+      <c r="F31" t="s">
+        <v>395</v>
+      </c>
+      <c r="G31" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>312</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C32" t="s">
+        <v>398</v>
+      </c>
+      <c r="D32" t="s">
+        <v>399</v>
+      </c>
+      <c r="G32" t="s">
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E7" r:id="rId1" xr:uid="{4D59EDE6-1E65-4897-A938-02BE975DD6E8}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3829A5A3-48FC-4C22-BABE-7F5589E4EDC1}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" customWidth="1"/>
+    <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
@@ -1146,7 +2294,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>75</v>
       </c>
@@ -1172,7 +2320,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>82</v>
       </c>
@@ -1198,7 +2346,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>87</v>
       </c>
@@ -1227,7 +2375,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -1256,7 +2404,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -1282,7 +2430,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>101</v>
       </c>
@@ -1308,7 +2456,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>105</v>
       </c>
@@ -1337,7 +2485,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -1366,7 +2514,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>115</v>
       </c>
@@ -1395,7 +2543,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>120</v>
       </c>
@@ -1421,7 +2569,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -1447,7 +2595,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>128</v>
       </c>
@@ -1455,7 +2603,7 @@
         <v>129</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>157</v>
+        <v>194</v>
       </c>
       <c r="E13" t="s">
         <v>91</v>
@@ -1473,7 +2621,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>131</v>
       </c>
@@ -1502,7 +2650,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>136</v>
       </c>
@@ -1531,7 +2679,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1560,7 +2708,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>146</v>
       </c>
@@ -1589,7 +2737,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>151</v>
       </c>
@@ -1618,10 +2766,732 @@
         <v>85</v>
       </c>
     </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B19" t="s">
+        <v>179</v>
+      </c>
+      <c r="C19" t="s">
+        <v>180</v>
+      </c>
+      <c r="D19" t="s">
+        <v>181</v>
+      </c>
+      <c r="E19" t="s">
+        <v>85</v>
+      </c>
+      <c r="F19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G19" t="s">
+        <v>80</v>
+      </c>
+      <c r="H19" t="s">
+        <v>160</v>
+      </c>
+      <c r="I19" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>183</v>
+      </c>
+      <c r="B20" t="s">
+        <v>184</v>
+      </c>
+      <c r="C20" t="s">
+        <v>185</v>
+      </c>
+      <c r="D20" t="s">
+        <v>186</v>
+      </c>
+      <c r="E20" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" t="s">
+        <v>187</v>
+      </c>
+      <c r="G20" t="s">
+        <v>114</v>
+      </c>
+      <c r="H20" t="s">
+        <v>188</v>
+      </c>
+      <c r="I20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>189</v>
+      </c>
+      <c r="B21" t="s">
+        <v>190</v>
+      </c>
+      <c r="C21" t="s">
+        <v>191</v>
+      </c>
+      <c r="D21" t="s">
+        <v>192</v>
+      </c>
+      <c r="E21" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" t="s">
+        <v>193</v>
+      </c>
+      <c r="G21" t="s">
+        <v>80</v>
+      </c>
+      <c r="H21" t="s">
+        <v>172</v>
+      </c>
+      <c r="I21" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>195</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C22" t="s">
+        <v>197</v>
+      </c>
+      <c r="D22" t="s">
+        <v>198</v>
+      </c>
+      <c r="E22" t="s">
+        <v>199</v>
+      </c>
+      <c r="F22" t="s">
+        <v>200</v>
+      </c>
+      <c r="G22" t="s">
+        <v>80</v>
+      </c>
+      <c r="H22" t="s">
+        <v>201</v>
+      </c>
+      <c r="I22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>202</v>
+      </c>
+      <c r="B23" t="s">
+        <v>203</v>
+      </c>
+      <c r="C23" t="s">
+        <v>204</v>
+      </c>
+      <c r="D23" t="s">
+        <v>205</v>
+      </c>
+      <c r="E23" t="s">
+        <v>85</v>
+      </c>
+      <c r="F23" t="s">
+        <v>206</v>
+      </c>
+      <c r="G23" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" t="s">
+        <v>7</v>
+      </c>
+      <c r="I23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B24" t="s">
+        <v>208</v>
+      </c>
+      <c r="C24" t="s">
+        <v>209</v>
+      </c>
+      <c r="D24" t="s">
+        <v>210</v>
+      </c>
+      <c r="E24" t="s">
+        <v>91</v>
+      </c>
+      <c r="F24" t="s">
+        <v>211</v>
+      </c>
+      <c r="G24" t="s">
+        <v>114</v>
+      </c>
+      <c r="H24" t="s">
+        <v>212</v>
+      </c>
+      <c r="I24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>213</v>
+      </c>
+      <c r="B25" t="s">
+        <v>214</v>
+      </c>
+      <c r="C25" t="s">
+        <v>215</v>
+      </c>
+      <c r="D25" t="s">
+        <v>216</v>
+      </c>
+      <c r="E25" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" t="s">
+        <v>217</v>
+      </c>
+      <c r="G25" t="s">
+        <v>114</v>
+      </c>
+      <c r="H25" t="s">
+        <v>218</v>
+      </c>
+      <c r="I25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" t="s">
+        <v>220</v>
+      </c>
+      <c r="C26" t="s">
+        <v>221</v>
+      </c>
+      <c r="D26" t="s">
+        <v>222</v>
+      </c>
+      <c r="E26" t="s">
+        <v>85</v>
+      </c>
+      <c r="F26" t="s">
+        <v>145</v>
+      </c>
+      <c r="G26" t="s">
+        <v>80</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>223</v>
+      </c>
+      <c r="B27" t="s">
+        <v>224</v>
+      </c>
+      <c r="C27" t="s">
+        <v>225</v>
+      </c>
+      <c r="D27" t="s">
+        <v>226</v>
+      </c>
+      <c r="E27" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" t="s">
+        <v>227</v>
+      </c>
+      <c r="G27" t="s">
+        <v>114</v>
+      </c>
+      <c r="H27" t="s">
+        <v>228</v>
+      </c>
+      <c r="I27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>229</v>
+      </c>
+      <c r="B28" t="s">
+        <v>230</v>
+      </c>
+      <c r="C28" t="s">
+        <v>231</v>
+      </c>
+      <c r="D28" t="s">
+        <v>232</v>
+      </c>
+      <c r="E28" t="s">
+        <v>91</v>
+      </c>
+      <c r="F28" t="s">
+        <v>233</v>
+      </c>
+      <c r="G28" t="s">
+        <v>80</v>
+      </c>
+      <c r="H28" t="s">
+        <v>234</v>
+      </c>
+      <c r="I28" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>235</v>
+      </c>
+      <c r="B29" t="s">
+        <v>236</v>
+      </c>
+      <c r="C29" t="s">
+        <v>237</v>
+      </c>
+      <c r="D29" t="s">
+        <v>238</v>
+      </c>
+      <c r="E29" t="s">
+        <v>239</v>
+      </c>
+      <c r="F29" t="s">
+        <v>240</v>
+      </c>
+      <c r="G29" t="s">
+        <v>80</v>
+      </c>
+      <c r="H29" t="s">
+        <v>228</v>
+      </c>
+      <c r="I29" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>241</v>
+      </c>
+      <c r="B30" t="s">
+        <v>242</v>
+      </c>
+      <c r="C30" t="s">
+        <v>243</v>
+      </c>
+      <c r="D30" t="s">
+        <v>244</v>
+      </c>
+      <c r="E30" t="s">
+        <v>85</v>
+      </c>
+      <c r="F30" t="s">
+        <v>104</v>
+      </c>
+      <c r="G30" t="s">
+        <v>80</v>
+      </c>
+      <c r="H30" t="s">
+        <v>7</v>
+      </c>
+      <c r="I30" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>245</v>
+      </c>
+      <c r="B31" t="s">
+        <v>246</v>
+      </c>
+      <c r="C31" t="s">
+        <v>247</v>
+      </c>
+      <c r="D31" t="s">
+        <v>248</v>
+      </c>
+      <c r="E31" t="s">
+        <v>85</v>
+      </c>
+      <c r="F31" t="s">
+        <v>249</v>
+      </c>
+      <c r="G31" t="s">
+        <v>80</v>
+      </c>
+      <c r="H31" t="s">
+        <v>250</v>
+      </c>
+      <c r="I31" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>251</v>
+      </c>
+      <c r="B32" t="s">
+        <v>252</v>
+      </c>
+      <c r="C32" t="s">
+        <v>253</v>
+      </c>
+      <c r="D32" t="s">
+        <v>254</v>
+      </c>
+      <c r="E32" t="s">
+        <v>78</v>
+      </c>
+      <c r="F32" t="s">
+        <v>255</v>
+      </c>
+      <c r="G32" t="s">
+        <v>80</v>
+      </c>
+      <c r="H32" t="s">
+        <v>256</v>
+      </c>
+      <c r="I32" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>257</v>
+      </c>
+      <c r="B33" t="s">
+        <v>258</v>
+      </c>
+      <c r="C33" t="s">
+        <v>259</v>
+      </c>
+      <c r="D33" t="s">
+        <v>260</v>
+      </c>
+      <c r="E33" t="s">
+        <v>261</v>
+      </c>
+      <c r="F33" t="s">
+        <v>127</v>
+      </c>
+      <c r="G33" t="s">
+        <v>114</v>
+      </c>
+      <c r="H33" t="s">
+        <v>262</v>
+      </c>
+      <c r="I33" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>263</v>
+      </c>
+      <c r="B34" t="s">
+        <v>264</v>
+      </c>
+      <c r="C34" t="s">
+        <v>215</v>
+      </c>
+      <c r="D34" t="s">
+        <v>265</v>
+      </c>
+      <c r="E34" t="s">
+        <v>261</v>
+      </c>
+      <c r="F34" t="s">
+        <v>266</v>
+      </c>
+      <c r="G34" t="s">
+        <v>80</v>
+      </c>
+      <c r="H34" t="s">
+        <v>262</v>
+      </c>
+      <c r="I34" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>267</v>
+      </c>
+      <c r="B35" t="s">
+        <v>268</v>
+      </c>
+      <c r="C35" t="s">
+        <v>269</v>
+      </c>
+      <c r="D35" t="s">
+        <v>270</v>
+      </c>
+      <c r="E35" t="s">
+        <v>85</v>
+      </c>
+      <c r="F35" t="s">
+        <v>271</v>
+      </c>
+      <c r="G35" t="s">
+        <v>114</v>
+      </c>
+      <c r="H35" t="s">
+        <v>272</v>
+      </c>
+      <c r="I35" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>273</v>
+      </c>
+      <c r="B36" t="s">
+        <v>274</v>
+      </c>
+      <c r="C36" t="s">
+        <v>275</v>
+      </c>
+      <c r="D36" t="s">
+        <v>276</v>
+      </c>
+      <c r="E36" t="s">
+        <v>85</v>
+      </c>
+      <c r="F36" t="s">
+        <v>277</v>
+      </c>
+      <c r="G36" t="s">
+        <v>80</v>
+      </c>
+      <c r="H36" t="s">
+        <v>278</v>
+      </c>
+      <c r="I36" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>279</v>
+      </c>
+      <c r="B37" t="s">
+        <v>280</v>
+      </c>
+      <c r="C37" t="s">
+        <v>281</v>
+      </c>
+      <c r="D37" t="s">
+        <v>282</v>
+      </c>
+      <c r="E37" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" t="s">
+        <v>283</v>
+      </c>
+      <c r="G37" t="s">
+        <v>114</v>
+      </c>
+      <c r="H37" t="s">
+        <v>284</v>
+      </c>
+      <c r="I37" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>285</v>
+      </c>
+      <c r="B38" t="s">
+        <v>286</v>
+      </c>
+      <c r="C38" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" t="s">
+        <v>288</v>
+      </c>
+      <c r="E38" t="s">
+        <v>91</v>
+      </c>
+      <c r="F38" t="s">
+        <v>289</v>
+      </c>
+      <c r="G38" t="s">
+        <v>114</v>
+      </c>
+      <c r="H38" t="s">
+        <v>290</v>
+      </c>
+      <c r="I38" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>291</v>
+      </c>
+      <c r="B39" t="s">
+        <v>292</v>
+      </c>
+      <c r="C39" t="s">
+        <v>215</v>
+      </c>
+      <c r="D39" t="s">
+        <v>293</v>
+      </c>
+      <c r="E39" t="s">
+        <v>85</v>
+      </c>
+      <c r="F39" t="s">
+        <v>294</v>
+      </c>
+      <c r="G39" t="s">
+        <v>80</v>
+      </c>
+      <c r="H39" t="s">
+        <v>295</v>
+      </c>
+      <c r="I39" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>296</v>
+      </c>
+      <c r="B40" t="s">
+        <v>297</v>
+      </c>
+      <c r="C40" t="s">
+        <v>298</v>
+      </c>
+      <c r="D40" t="s">
+        <v>299</v>
+      </c>
+      <c r="E40" t="s">
+        <v>85</v>
+      </c>
+      <c r="F40" t="s">
+        <v>294</v>
+      </c>
+      <c r="G40" t="s">
+        <v>80</v>
+      </c>
+      <c r="H40" t="s">
+        <v>300</v>
+      </c>
+      <c r="I40" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>301</v>
+      </c>
+      <c r="B41" t="s">
+        <v>302</v>
+      </c>
+      <c r="C41" t="s">
+        <v>303</v>
+      </c>
+      <c r="D41" t="s">
+        <v>304</v>
+      </c>
+      <c r="E41" t="s">
+        <v>199</v>
+      </c>
+      <c r="F41" t="s">
+        <v>305</v>
+      </c>
+      <c r="G41" t="s">
+        <v>114</v>
+      </c>
+      <c r="H41" t="s">
+        <v>306</v>
+      </c>
+      <c r="I41" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>307</v>
+      </c>
+      <c r="B42" t="s">
+        <v>308</v>
+      </c>
+      <c r="C42" t="s">
+        <v>309</v>
+      </c>
+      <c r="D42" t="s">
+        <v>310</v>
+      </c>
+      <c r="E42" t="s">
+        <v>78</v>
+      </c>
+      <c r="F42" t="s">
+        <v>311</v>
+      </c>
+      <c r="G42" t="s">
+        <v>114</v>
+      </c>
+      <c r="H42" t="s">
+        <v>312</v>
+      </c>
+      <c r="I42" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>313</v>
+      </c>
+      <c r="B43" t="s">
+        <v>314</v>
+      </c>
+      <c r="C43" t="s">
+        <v>315</v>
+      </c>
+      <c r="D43" t="s">
+        <v>316</v>
+      </c>
+      <c r="E43" t="s">
+        <v>199</v>
+      </c>
+      <c r="F43" t="s">
+        <v>127</v>
+      </c>
+      <c r="G43" t="s">
+        <v>114</v>
+      </c>
+      <c r="H43" t="s">
+        <v>201</v>
+      </c>
+      <c r="I43" t="s">
+        <v>199</v>
+      </c>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D13" r:id="rId1" xr:uid="{1D3AF0E2-67F2-4181-94BE-6DFCC04AD494}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>